<commit_message>
Corrida | SFE-SUP | 2026-06-17 11:33:26.953778
</commit_message>
<xml_diff>
--- a/indicadores/SFE-SUP_out.xlsx
+++ b/indicadores/SFE-SUP_out.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="572">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="574">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -23,7 +23,7 @@
     <t xml:space="preserve">Título</t>
   </si>
   <si>
-    <t xml:space="preserve">Superficie cubierta autorizada en algunos municipios de la provincia de Santa Fe</t>
+    <t xml:space="preserve">Superficie cubierta autorizada</t>
   </si>
   <si>
     <t xml:space="preserve">Unidad de medida</t>
@@ -74,6 +74,12 @@
     <t xml:space="preserve">const</t>
   </si>
   <si>
+    <t xml:space="preserve">Alcance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provincia de Santa Fe</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumen del correlograma</t>
   </si>
   <si>
@@ -107,13 +113,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">01/06/2026</t>
+    <t xml:space="preserve">17/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">ysonder</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -2232,9 +2238,13 @@
       <c r="J6" s="1"/>
     </row>
     <row r="7">
-      <c r="A7"/>
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
       <c r="B7"/>
-      <c r="C7"/>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7"/>
@@ -2245,7 +2255,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B8"/>
       <c r="C8"/>
@@ -2259,7 +2269,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B9"/>
       <c r="C9"/>
@@ -2275,7 +2285,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
@@ -2303,7 +2313,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B12"/>
       <c r="C12"/>
@@ -2317,7 +2327,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B13"/>
       <c r="C13"/>
@@ -2345,7 +2355,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
@@ -2359,7 +2369,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B16"/>
       <c r="C16"/>
@@ -2373,7 +2383,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -2387,7 +2397,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
@@ -2403,7 +2413,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -2417,7 +2427,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B20"/>
       <c r="C20"/>
@@ -2565,10 +2575,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C32"/>
       <c r="D32"/>
@@ -2581,10 +2591,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B33" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C33"/>
       <c r="D33"/>
@@ -2608,66 +2618,66 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="I1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="K1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="M1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="N1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="O1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="P1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="Q1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="R1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="S1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>8.431</v>
@@ -2720,7 +2730,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>9.898</v>
@@ -2777,7 +2787,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>11.888</v>
@@ -2834,7 +2844,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>9.238</v>
@@ -2891,7 +2901,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>14.1</v>
@@ -2948,7 +2958,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>11.147</v>
@@ -3005,7 +3015,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>15.338</v>
@@ -3062,7 +3072,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>18.407</v>
@@ -3119,7 +3129,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>18.113</v>
@@ -3176,7 +3186,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>22.971</v>
@@ -3233,7 +3243,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>27.928</v>
@@ -3290,7 +3300,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>19.228</v>
@@ -3347,7 +3357,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>7.932</v>
@@ -3406,7 +3416,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>9.541</v>
@@ -3465,7 +3475,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>20.106</v>
@@ -3524,7 +3534,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>17.017</v>
@@ -3583,7 +3593,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>17.228</v>
@@ -3642,7 +3652,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>20.847</v>
@@ -3701,7 +3711,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>15.915</v>
@@ -3760,7 +3770,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>21.987</v>
@@ -3819,7 +3829,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>34.949</v>
@@ -3878,7 +3888,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>27.792</v>
@@ -3937,7 +3947,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>23.862</v>
@@ -3996,7 +4006,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>19.086</v>
@@ -4055,7 +4065,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>15.738</v>
@@ -4114,7 +4124,7 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>34.781</v>
@@ -4173,7 +4183,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>31.931</v>
@@ -4232,7 +4242,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>34.091</v>
@@ -4291,7 +4301,7 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>23.215</v>
@@ -4350,7 +4360,7 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>28.471</v>
@@ -4409,7 +4419,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>23.297</v>
@@ -4468,7 +4478,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>31.023</v>
@@ -4527,7 +4537,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>32.377</v>
@@ -4586,7 +4596,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>32.742</v>
@@ -4645,7 +4655,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>39.817</v>
@@ -4704,7 +4714,7 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>31.972</v>
@@ -4763,7 +4773,7 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>21.605</v>
@@ -4822,7 +4832,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>37.3</v>
@@ -4881,7 +4891,7 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B40" s="2" t="n">
         <v>69.572</v>
@@ -4940,7 +4950,7 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B41" s="2" t="n">
         <v>64.302</v>
@@ -4999,7 +5009,7 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B42" s="2" t="n">
         <v>63.165</v>
@@ -5058,7 +5068,7 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B43" s="2" t="n">
         <v>60.464</v>
@@ -5117,7 +5127,7 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B44" s="2" t="n">
         <v>67.614</v>
@@ -5176,7 +5186,7 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B45" s="2" t="n">
         <v>45.516</v>
@@ -5235,7 +5245,7 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B46" s="2" t="n">
         <v>46.277</v>
@@ -5294,7 +5304,7 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B47" s="2" t="n">
         <v>39.536</v>
@@ -5353,7 +5363,7 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B48" s="2" t="n">
         <v>46.824</v>
@@ -5412,7 +5422,7 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B49" s="2" t="n">
         <v>39.203</v>
@@ -5471,7 +5481,7 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B50" s="2" t="n">
         <v>26.741</v>
@@ -5530,7 +5540,7 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B51" s="2" t="n">
         <v>32.765</v>
@@ -5589,7 +5599,7 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B52" s="2" t="n">
         <v>46.212</v>
@@ -5648,7 +5658,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B53" s="2" t="n">
         <v>33.729</v>
@@ -5707,7 +5717,7 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B54" s="2" t="n">
         <v>35.933</v>
@@ -5766,7 +5776,7 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B55" s="2" t="n">
         <v>45.48</v>
@@ -5825,7 +5835,7 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B56" s="2" t="n">
         <v>26.406</v>
@@ -5884,7 +5894,7 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B57" s="2" t="n">
         <v>37.693</v>
@@ -5943,7 +5953,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B58" s="2" t="n">
         <v>26.201</v>
@@ -6002,7 +6012,7 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B59" s="2" t="n">
         <v>33.929</v>
@@ -6061,7 +6071,7 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B60" s="2" t="n">
         <v>31.173</v>
@@ -6120,7 +6130,7 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B61" s="2" t="n">
         <v>35.128</v>
@@ -6179,7 +6189,7 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B62" s="2" t="n">
         <v>13.474</v>
@@ -6238,7 +6248,7 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B63" s="2" t="n">
         <v>22.139</v>
@@ -6297,7 +6307,7 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B64" s="2" t="n">
         <v>25.539</v>
@@ -6356,7 +6366,7 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B65" s="2" t="n">
         <v>26.089</v>
@@ -6415,7 +6425,7 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B66" s="2" t="n">
         <v>26.863</v>
@@ -6474,7 +6484,7 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B67" s="2" t="n">
         <v>27.245</v>
@@ -6533,7 +6543,7 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B68" s="2" t="n">
         <v>29.715</v>
@@ -6592,7 +6602,7 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B69" s="2" t="n">
         <v>42.813</v>
@@ -6651,7 +6661,7 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B70" s="2" t="n">
         <v>37.27</v>
@@ -6710,7 +6720,7 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B71" s="2" t="n">
         <v>42.856</v>
@@ -6769,7 +6779,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B72" s="2" t="n">
         <v>40.159</v>
@@ -6828,7 +6838,7 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B73" s="2" t="n">
         <v>35.428</v>
@@ -6887,7 +6897,7 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B74" s="2" t="n">
         <v>48.45</v>
@@ -6946,7 +6956,7 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B75" s="2" t="n">
         <v>15.023</v>
@@ -7005,7 +7015,7 @@
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B76" s="2" t="n">
         <v>32.864</v>
@@ -7064,7 +7074,7 @@
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B77" s="2" t="n">
         <v>34.964</v>
@@ -7123,7 +7133,7 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B78" s="2" t="n">
         <v>29.35</v>
@@ -7182,7 +7192,7 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B79" s="2" t="n">
         <v>28.562</v>
@@ -7241,7 +7251,7 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B80" s="2" t="n">
         <v>31.512</v>
@@ -7300,7 +7310,7 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B81" s="2" t="n">
         <v>22.15</v>
@@ -7359,7 +7369,7 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B82" s="2" t="n">
         <v>51.412</v>
@@ -7418,7 +7428,7 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B83" s="2" t="n">
         <v>39.889</v>
@@ -7477,7 +7487,7 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B84" s="2" t="n">
         <v>39.943</v>
@@ -7536,7 +7546,7 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B85" s="2" t="n">
         <v>31.246</v>
@@ -7595,7 +7605,7 @@
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B86" s="2" t="n">
         <v>32.797</v>
@@ -7654,7 +7664,7 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B87" s="2" t="n">
         <v>24.646</v>
@@ -7713,7 +7723,7 @@
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B88" s="2" t="n">
         <v>37.244</v>
@@ -7772,7 +7782,7 @@
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B89" s="2" t="n">
         <v>37.21</v>
@@ -7831,7 +7841,7 @@
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B90" s="2" t="n">
         <v>40.285</v>
@@ -7890,7 +7900,7 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B91" s="2" t="n">
         <v>60.066</v>
@@ -7949,7 +7959,7 @@
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B92" s="2" t="n">
         <v>42.232</v>
@@ -8008,7 +8018,7 @@
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B93" s="2" t="n">
         <v>37.357</v>
@@ -8067,7 +8077,7 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B94" s="2" t="n">
         <v>48.68</v>
@@ -8126,7 +8136,7 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B95" s="2" t="n">
         <v>39.28</v>
@@ -8185,7 +8195,7 @@
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B96" s="2" t="n">
         <v>37.8</v>
@@ -8244,7 +8254,7 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B97" s="2" t="n">
         <v>43.984</v>
@@ -8303,7 +8313,7 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B98" s="2" t="n">
         <v>26.726</v>
@@ -8362,7 +8372,7 @@
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B99" s="2" t="n">
         <v>42.564</v>
@@ -8421,7 +8431,7 @@
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B100" s="2" t="n">
         <v>48.751</v>
@@ -8480,7 +8490,7 @@
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B101" s="2" t="n">
         <v>41.868</v>
@@ -8539,7 +8549,7 @@
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B102" s="2" t="n">
         <v>29.668</v>
@@ -8598,7 +8608,7 @@
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B103" s="2" t="n">
         <v>54.892</v>
@@ -8657,7 +8667,7 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B104" s="2" t="n">
         <v>43.603</v>
@@ -8716,7 +8726,7 @@
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B105" s="2" t="n">
         <v>44.231</v>
@@ -8775,7 +8785,7 @@
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B106" s="2" t="n">
         <v>53.979</v>
@@ -8834,7 +8844,7 @@
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B107" s="2" t="n">
         <v>43.932</v>
@@ -8893,7 +8903,7 @@
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B108" s="2" t="n">
         <v>37.535</v>
@@ -8952,7 +8962,7 @@
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B109" s="2" t="n">
         <v>55.76</v>
@@ -9011,7 +9021,7 @@
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B110" s="2" t="n">
         <v>28.736</v>
@@ -9070,7 +9080,7 @@
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B111" s="2" t="n">
         <v>33.267</v>
@@ -9129,7 +9139,7 @@
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B112" s="2" t="n">
         <v>42.497</v>
@@ -9188,7 +9198,7 @@
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B113" s="2" t="n">
         <v>30.977</v>
@@ -9247,7 +9257,7 @@
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B114" s="2" t="n">
         <v>39.395</v>
@@ -9306,7 +9316,7 @@
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B115" s="2" t="n">
         <v>30.38</v>
@@ -9365,7 +9375,7 @@
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B116" s="2" t="n">
         <v>32.22</v>
@@ -9424,7 +9434,7 @@
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B117" s="2" t="n">
         <v>42.538</v>
@@ -9483,7 +9493,7 @@
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B118" s="2" t="n">
         <v>33.25</v>
@@ -9542,7 +9552,7 @@
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B119" s="2" t="n">
         <v>31.583</v>
@@ -9601,7 +9611,7 @@
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B120" s="2" t="n">
         <v>28.229</v>
@@ -9660,7 +9670,7 @@
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B121" s="2" t="n">
         <v>34.672</v>
@@ -9719,7 +9729,7 @@
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B122" s="2" t="n">
         <v>23.065</v>
@@ -9778,7 +9788,7 @@
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B123" s="2" t="n">
         <v>37.057</v>
@@ -9837,7 +9847,7 @@
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B124" s="2" t="n">
         <v>36.377</v>
@@ -9896,7 +9906,7 @@
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B125" s="2" t="n">
         <v>27.834</v>
@@ -9955,7 +9965,7 @@
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B126" s="2" t="n">
         <v>43.657</v>
@@ -10014,7 +10024,7 @@
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B127" s="2" t="n">
         <v>31.409</v>
@@ -10073,7 +10083,7 @@
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B128" s="2" t="n">
         <v>34.477</v>
@@ -10132,7 +10142,7 @@
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B129" s="2" t="n">
         <v>32.884</v>
@@ -10191,7 +10201,7 @@
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B130" s="2" t="n">
         <v>47.654</v>
@@ -10250,7 +10260,7 @@
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B131" s="2" t="n">
         <v>28.465</v>
@@ -10309,7 +10319,7 @@
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B132" s="2" t="n">
         <v>27.131</v>
@@ -10368,7 +10378,7 @@
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B133" s="2" t="n">
         <v>24.333</v>
@@ -10427,7 +10437,7 @@
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B134" s="2" t="n">
         <v>9.877</v>
@@ -10486,7 +10496,7 @@
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B135" s="2" t="n">
         <v>31.46</v>
@@ -10545,7 +10555,7 @@
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B136" s="2" t="n">
         <v>22.547</v>
@@ -10604,7 +10614,7 @@
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B137" s="2" t="n">
         <v>23.248</v>
@@ -10663,7 +10673,7 @@
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B138" s="2" t="n">
         <v>32.158</v>
@@ -10722,7 +10732,7 @@
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B139" s="2" t="n">
         <v>29.718</v>
@@ -10781,7 +10791,7 @@
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B140" s="2" t="n">
         <v>26.917</v>
@@ -10840,7 +10850,7 @@
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B141" s="2" t="n">
         <v>35.791</v>
@@ -10899,7 +10909,7 @@
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B142" s="2" t="n">
         <v>33.98</v>
@@ -10958,7 +10968,7 @@
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B143" s="2" t="n">
         <v>32.654</v>
@@ -11017,7 +11027,7 @@
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B144" s="2" t="n">
         <v>31.775</v>
@@ -11076,7 +11086,7 @@
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B145" s="2" t="n">
         <v>43.8</v>
@@ -11135,7 +11145,7 @@
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B146" s="2" t="n">
         <v>14.85</v>
@@ -11194,7 +11204,7 @@
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B147" s="2" t="n">
         <v>34.272</v>
@@ -11253,7 +11263,7 @@
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B148" s="2" t="n">
         <v>36.94</v>
@@ -11312,7 +11322,7 @@
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B149" s="2" t="n">
         <v>37.995</v>
@@ -11371,7 +11381,7 @@
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B150" s="2" t="n">
         <v>25.266</v>
@@ -11430,7 +11440,7 @@
     </row>
     <row r="151">
       <c r="A151" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B151" s="2" t="n">
         <v>31.241</v>
@@ -11489,7 +11499,7 @@
     </row>
     <row r="152">
       <c r="A152" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B152" s="2" t="n">
         <v>32.613</v>
@@ -11548,7 +11558,7 @@
     </row>
     <row r="153">
       <c r="A153" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B153" s="2" t="n">
         <v>25.028</v>
@@ -11607,7 +11617,7 @@
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B154" s="2" t="n">
         <v>38.775</v>
@@ -11666,7 +11676,7 @@
     </row>
     <row r="155">
       <c r="A155" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B155" s="2" t="n">
         <v>37.775</v>
@@ -11725,7 +11735,7 @@
     </row>
     <row r="156">
       <c r="A156" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B156" s="2" t="n">
         <v>33.915</v>
@@ -11784,7 +11794,7 @@
     </row>
     <row r="157">
       <c r="A157" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B157" s="2" t="n">
         <v>33.785</v>
@@ -11843,7 +11853,7 @@
     </row>
     <row r="158">
       <c r="A158" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B158" s="2" t="n">
         <v>13.76</v>
@@ -11902,7 +11912,7 @@
     </row>
     <row r="159">
       <c r="A159" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B159" s="2" t="n">
         <v>28.685</v>
@@ -11961,7 +11971,7 @@
     </row>
     <row r="160">
       <c r="A160" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B160" s="2" t="n">
         <v>36.061</v>
@@ -12020,7 +12030,7 @@
     </row>
     <row r="161">
       <c r="A161" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B161" s="2" t="n">
         <v>27.61</v>
@@ -12079,7 +12089,7 @@
     </row>
     <row r="162">
       <c r="A162" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B162" s="2" t="n">
         <v>36.109</v>
@@ -12138,7 +12148,7 @@
     </row>
     <row r="163">
       <c r="A163" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B163" s="2" t="n">
         <v>35.944</v>
@@ -12197,7 +12207,7 @@
     </row>
     <row r="164">
       <c r="A164" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B164" s="2" t="n">
         <v>42.977</v>
@@ -12256,7 +12266,7 @@
     </row>
     <row r="165">
       <c r="A165" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B165" s="2" t="n">
         <v>48.826</v>
@@ -12315,7 +12325,7 @@
     </row>
     <row r="166">
       <c r="A166" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B166" s="2" t="n">
         <v>52.392</v>
@@ -12374,7 +12384,7 @@
     </row>
     <row r="167">
       <c r="A167" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B167" s="2" t="n">
         <v>42.62</v>
@@ -12433,7 +12443,7 @@
     </row>
     <row r="168">
       <c r="A168" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B168" s="2" t="n">
         <v>35.631</v>
@@ -12492,7 +12502,7 @@
     </row>
     <row r="169">
       <c r="A169" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B169" s="2" t="n">
         <v>46.055</v>
@@ -12551,7 +12561,7 @@
     </row>
     <row r="170">
       <c r="A170" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B170" s="2" t="n">
         <v>27.226</v>
@@ -12610,7 +12620,7 @@
     </row>
     <row r="171">
       <c r="A171" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B171" s="2" t="n">
         <v>26.686</v>
@@ -12669,7 +12679,7 @@
     </row>
     <row r="172">
       <c r="A172" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B172" s="2" t="n">
         <v>46.409</v>
@@ -12728,7 +12738,7 @@
     </row>
     <row r="173">
       <c r="A173" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B173" s="2" t="n">
         <v>48.331</v>
@@ -12787,7 +12797,7 @@
     </row>
     <row r="174">
       <c r="A174" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B174" s="2" t="n">
         <v>51.642</v>
@@ -12846,7 +12856,7 @@
     </row>
     <row r="175">
       <c r="A175" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B175" s="2" t="n">
         <v>58.999</v>
@@ -12905,7 +12915,7 @@
     </row>
     <row r="176">
       <c r="A176" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B176" s="2" t="n">
         <v>47.581</v>
@@ -12964,7 +12974,7 @@
     </row>
     <row r="177">
       <c r="A177" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B177" s="2" t="n">
         <v>54.179</v>
@@ -13023,7 +13033,7 @@
     </row>
     <row r="178">
       <c r="A178" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B178" s="2" t="n">
         <v>52.27</v>
@@ -13082,7 +13092,7 @@
     </row>
     <row r="179">
       <c r="A179" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B179" s="2" t="n">
         <v>57.684</v>
@@ -13141,7 +13151,7 @@
     </row>
     <row r="180">
       <c r="A180" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B180" s="2" t="n">
         <v>56.13</v>
@@ -13200,7 +13210,7 @@
     </row>
     <row r="181">
       <c r="A181" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B181" s="2" t="n">
         <v>66.538</v>
@@ -13259,7 +13269,7 @@
     </row>
     <row r="182">
       <c r="A182" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B182" s="2" t="n">
         <v>22.568</v>
@@ -13318,7 +13328,7 @@
     </row>
     <row r="183">
       <c r="A183" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B183" s="2" t="n">
         <v>57.409</v>
@@ -13377,7 +13387,7 @@
     </row>
     <row r="184">
       <c r="A184" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B184" s="2" t="n">
         <v>43.004</v>
@@ -13436,7 +13446,7 @@
     </row>
     <row r="185">
       <c r="A185" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B185" s="2" t="n">
         <v>46.578</v>
@@ -13495,7 +13505,7 @@
     </row>
     <row r="186">
       <c r="A186" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B186" s="2" t="n">
         <v>82.015</v>
@@ -13554,7 +13564,7 @@
     </row>
     <row r="187">
       <c r="A187" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B187" s="2" t="n">
         <v>70.939</v>
@@ -13613,7 +13623,7 @@
     </row>
     <row r="188">
       <c r="A188" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B188" s="2" t="n">
         <v>46.449</v>
@@ -13672,7 +13682,7 @@
     </row>
     <row r="189">
       <c r="A189" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B189" s="2" t="n">
         <v>54.56</v>
@@ -13731,7 +13741,7 @@
     </row>
     <row r="190">
       <c r="A190" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B190" s="2" t="n">
         <v>65.935</v>
@@ -13790,7 +13800,7 @@
     </row>
     <row r="191">
       <c r="A191" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B191" s="2" t="n">
         <v>56.105</v>
@@ -13849,7 +13859,7 @@
     </row>
     <row r="192">
       <c r="A192" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B192" s="2" t="n">
         <v>65.002</v>
@@ -13908,7 +13918,7 @@
     </row>
     <row r="193">
       <c r="A193" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B193" s="2" t="n">
         <v>82.724</v>
@@ -13967,7 +13977,7 @@
     </row>
     <row r="194">
       <c r="A194" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B194" s="2" t="n">
         <v>32.791</v>
@@ -14026,7 +14036,7 @@
     </row>
     <row r="195">
       <c r="A195" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B195" s="2" t="n">
         <v>56.958</v>
@@ -14085,7 +14095,7 @@
     </row>
     <row r="196">
       <c r="A196" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B196" s="2" t="n">
         <v>76.006</v>
@@ -14144,7 +14154,7 @@
     </row>
     <row r="197">
       <c r="A197" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B197" s="2" t="n">
         <v>58.565</v>
@@ -14203,7 +14213,7 @@
     </row>
     <row r="198">
       <c r="A198" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B198" s="2" t="n">
         <v>73.458</v>
@@ -14262,7 +14272,7 @@
     </row>
     <row r="199">
       <c r="A199" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B199" s="2" t="n">
         <v>63.12</v>
@@ -14321,7 +14331,7 @@
     </row>
     <row r="200">
       <c r="A200" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B200" s="2" t="n">
         <v>51.518</v>
@@ -14380,7 +14390,7 @@
     </row>
     <row r="201">
       <c r="A201" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B201" s="2" t="n">
         <v>56.937</v>
@@ -14439,7 +14449,7 @@
     </row>
     <row r="202">
       <c r="A202" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B202" s="2" t="n">
         <v>65.713</v>
@@ -14498,7 +14508,7 @@
     </row>
     <row r="203">
       <c r="A203" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B203" s="2" t="n">
         <v>71.65</v>
@@ -14557,7 +14567,7 @@
     </row>
     <row r="204">
       <c r="A204" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B204" s="2" t="n">
         <v>66.733</v>
@@ -14616,7 +14626,7 @@
     </row>
     <row r="205">
       <c r="A205" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B205" s="2" t="n">
         <v>62.737</v>
@@ -14675,7 +14685,7 @@
     </row>
     <row r="206">
       <c r="A206" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B206" s="2" t="n">
         <v>53.867</v>
@@ -14734,7 +14744,7 @@
     </row>
     <row r="207">
       <c r="A207" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B207" s="2" t="n">
         <v>48.054</v>
@@ -14793,7 +14803,7 @@
     </row>
     <row r="208">
       <c r="A208" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B208" s="2" t="n">
         <v>77.194</v>
@@ -14852,7 +14862,7 @@
     </row>
     <row r="209">
       <c r="A209" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B209" s="2" t="n">
         <v>60.29</v>
@@ -14911,7 +14921,7 @@
     </row>
     <row r="210">
       <c r="A210" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B210" s="2" t="n">
         <v>64.747</v>
@@ -14970,7 +14980,7 @@
     </row>
     <row r="211">
       <c r="A211" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B211" s="2" t="n">
         <v>65.676</v>
@@ -15029,7 +15039,7 @@
     </row>
     <row r="212">
       <c r="A212" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B212" s="2" t="n">
         <v>75.371</v>
@@ -15088,7 +15098,7 @@
     </row>
     <row r="213">
       <c r="A213" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B213" s="2" t="n">
         <v>92.033</v>
@@ -15147,7 +15157,7 @@
     </row>
     <row r="214">
       <c r="A214" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B214" s="2" t="n">
         <v>98.715</v>
@@ -15206,7 +15216,7 @@
     </row>
     <row r="215">
       <c r="A215" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B215" s="2" t="n">
         <v>58.929</v>
@@ -15265,7 +15275,7 @@
     </row>
     <row r="216">
       <c r="A216" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B216" s="2" t="n">
         <v>85.191</v>
@@ -15324,7 +15334,7 @@
     </row>
     <row r="217">
       <c r="A217" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B217" s="2" t="n">
         <v>63.554</v>
@@ -15383,7 +15393,7 @@
     </row>
     <row r="218">
       <c r="A218" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B218" s="2" t="n">
         <v>33.813</v>
@@ -15442,7 +15452,7 @@
     </row>
     <row r="219">
       <c r="A219" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B219" s="2" t="n">
         <v>21.955</v>
@@ -15501,7 +15511,7 @@
     </row>
     <row r="220">
       <c r="A220" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B220" s="2" t="n">
         <v>69.46</v>
@@ -15560,7 +15570,7 @@
     </row>
     <row r="221">
       <c r="A221" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B221" s="2" t="n">
         <v>70.869</v>
@@ -15619,7 +15629,7 @@
     </row>
     <row r="222">
       <c r="A222" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B222" s="2" t="n">
         <v>41.684</v>
@@ -15678,7 +15688,7 @@
     </row>
     <row r="223">
       <c r="A223" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B223" s="2" t="n">
         <v>51.766</v>
@@ -15737,7 +15747,7 @@
     </row>
     <row r="224">
       <c r="A224" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B224" s="2" t="n">
         <v>51.914</v>
@@ -15796,7 +15806,7 @@
     </row>
     <row r="225">
       <c r="A225" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B225" s="2" t="n">
         <v>52.615</v>
@@ -15855,7 +15865,7 @@
     </row>
     <row r="226">
       <c r="A226" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B226" s="2" t="n">
         <v>68.997</v>
@@ -15914,7 +15924,7 @@
     </row>
     <row r="227">
       <c r="A227" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B227" s="2" t="n">
         <v>68.39</v>
@@ -15973,7 +15983,7 @@
     </row>
     <row r="228">
       <c r="A228" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B228" s="2" t="n">
         <v>77.65</v>
@@ -16032,7 +16042,7 @@
     </row>
     <row r="229">
       <c r="A229" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B229" s="2" t="n">
         <v>74.01</v>
@@ -16091,7 +16101,7 @@
     </row>
     <row r="230">
       <c r="A230" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B230" s="2" t="n">
         <v>53.442</v>
@@ -16150,7 +16160,7 @@
     </row>
     <row r="231">
       <c r="A231" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B231" s="2" t="n">
         <v>50.203</v>
@@ -16209,7 +16219,7 @@
     </row>
     <row r="232">
       <c r="A232" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B232" s="2" t="n">
         <v>51.369</v>
@@ -16268,7 +16278,7 @@
     </row>
     <row r="233">
       <c r="A233" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B233" s="2" t="n">
         <v>70.845</v>
@@ -16327,7 +16337,7 @@
     </row>
     <row r="234">
       <c r="A234" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B234" s="2" t="n">
         <v>63.18</v>
@@ -16386,7 +16396,7 @@
     </row>
     <row r="235">
       <c r="A235" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B235" s="2" t="n">
         <v>84.032</v>
@@ -16445,7 +16455,7 @@
     </row>
     <row r="236">
       <c r="A236" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B236" s="2" t="n">
         <v>105.587</v>
@@ -16504,7 +16514,7 @@
     </row>
     <row r="237">
       <c r="A237" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B237" s="2" t="n">
         <v>97.028</v>
@@ -16563,7 +16573,7 @@
     </row>
     <row r="238">
       <c r="A238" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B238" s="2" t="n">
         <v>72.051</v>
@@ -16622,7 +16632,7 @@
     </row>
     <row r="239">
       <c r="A239" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B239" s="2" t="n">
         <v>57.229</v>
@@ -16681,7 +16691,7 @@
     </row>
     <row r="240">
       <c r="A240" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B240" s="2" t="n">
         <v>57.468</v>
@@ -16740,7 +16750,7 @@
     </row>
     <row r="241">
       <c r="A241" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B241" s="2" t="n">
         <v>88.419</v>
@@ -16799,7 +16809,7 @@
     </row>
     <row r="242">
       <c r="A242" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B242" s="2" t="n">
         <v>45.63</v>
@@ -16858,7 +16868,7 @@
     </row>
     <row r="243">
       <c r="A243" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B243" s="2" t="n">
         <v>55.863</v>
@@ -16917,7 +16927,7 @@
     </row>
     <row r="244">
       <c r="A244" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B244" s="2" t="n">
         <v>64.097</v>
@@ -16976,7 +16986,7 @@
     </row>
     <row r="245">
       <c r="A245" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B245" s="2" t="n">
         <v>71.607</v>
@@ -17035,7 +17045,7 @@
     </row>
     <row r="246">
       <c r="A246" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B246" s="2" t="n">
         <v>82.235</v>
@@ -17094,7 +17104,7 @@
     </row>
     <row r="247">
       <c r="A247" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B247" s="2" t="n">
         <v>55.656</v>
@@ -17153,7 +17163,7 @@
     </row>
     <row r="248">
       <c r="A248" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B248" s="2" t="n">
         <v>53.827</v>
@@ -17212,7 +17222,7 @@
     </row>
     <row r="249">
       <c r="A249" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B249" s="2" t="n">
         <v>90.912</v>
@@ -17271,7 +17281,7 @@
     </row>
     <row r="250">
       <c r="A250" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B250" s="2" t="n">
         <v>96.959</v>
@@ -17330,7 +17340,7 @@
     </row>
     <row r="251">
       <c r="A251" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B251" s="2" t="n">
         <v>70.58</v>
@@ -17389,7 +17399,7 @@
     </row>
     <row r="252">
       <c r="A252" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B252" s="2" t="n">
         <v>85.449</v>
@@ -17448,7 +17458,7 @@
     </row>
     <row r="253">
       <c r="A253" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B253" s="2" t="n">
         <v>66.643</v>
@@ -17507,7 +17517,7 @@
     </row>
     <row r="254">
       <c r="A254" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B254" s="2" t="n">
         <v>47.511</v>
@@ -17566,7 +17576,7 @@
     </row>
     <row r="255">
       <c r="A255" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B255" s="2" t="n">
         <v>49.623</v>
@@ -17625,7 +17635,7 @@
     </row>
     <row r="256">
       <c r="A256" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B256" s="2" t="n">
         <v>44.999</v>
@@ -17684,7 +17694,7 @@
     </row>
     <row r="257">
       <c r="A257" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B257" s="2" t="n">
         <v>65.935</v>
@@ -17743,7 +17753,7 @@
     </row>
     <row r="258">
       <c r="A258" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B258" s="2" t="n">
         <v>74.348</v>
@@ -17802,7 +17812,7 @@
     </row>
     <row r="259">
       <c r="A259" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B259" s="2" t="n">
         <v>58.622</v>
@@ -17861,7 +17871,7 @@
     </row>
     <row r="260">
       <c r="A260" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B260" s="2" t="n">
         <v>66.073</v>
@@ -17920,7 +17930,7 @@
     </row>
     <row r="261">
       <c r="A261" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B261" s="2" t="n">
         <v>116.609</v>
@@ -17979,7 +17989,7 @@
     </row>
     <row r="262">
       <c r="A262" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B262" s="2" t="n">
         <v>81.855</v>
@@ -18038,7 +18048,7 @@
     </row>
     <row r="263">
       <c r="A263" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B263" s="2" t="n">
         <v>58.537</v>
@@ -18097,7 +18107,7 @@
     </row>
     <row r="264">
       <c r="A264" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B264" s="2" t="n">
         <v>61.645</v>
@@ -18156,7 +18166,7 @@
     </row>
     <row r="265">
       <c r="A265" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B265" s="2" t="n">
         <v>44.185</v>
@@ -18215,7 +18225,7 @@
     </row>
     <row r="266">
       <c r="A266" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B266" s="2" t="n">
         <v>57.041</v>
@@ -18274,7 +18284,7 @@
     </row>
     <row r="267">
       <c r="A267" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B267" s="2" t="n">
         <v>54.17</v>
@@ -18333,7 +18343,7 @@
     </row>
     <row r="268">
       <c r="A268" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B268" s="2" t="n">
         <v>68.088</v>
@@ -18392,7 +18402,7 @@
     </row>
     <row r="269">
       <c r="A269" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B269" s="2" t="n">
         <v>71.988</v>
@@ -18451,7 +18461,7 @@
     </row>
     <row r="270">
       <c r="A270" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B270" s="2" t="n">
         <v>71.063</v>
@@ -18510,7 +18520,7 @@
     </row>
     <row r="271">
       <c r="A271" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B271" s="2" t="n">
         <v>64.065</v>
@@ -18569,7 +18579,7 @@
     </row>
     <row r="272">
       <c r="A272" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B272" s="2" t="n">
         <v>71.783</v>
@@ -18628,7 +18638,7 @@
     </row>
     <row r="273">
       <c r="A273" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B273" s="2" t="n">
         <v>73.847</v>
@@ -18687,7 +18697,7 @@
     </row>
     <row r="274">
       <c r="A274" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B274" s="2" t="n">
         <v>79.178</v>
@@ -18746,7 +18756,7 @@
     </row>
     <row r="275">
       <c r="A275" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B275" s="2" t="n">
         <v>75.087</v>
@@ -18805,7 +18815,7 @@
     </row>
     <row r="276">
       <c r="A276" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B276" s="2" t="n">
         <v>65.072</v>
@@ -18864,7 +18874,7 @@
     </row>
     <row r="277">
       <c r="A277" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B277" s="2" t="n">
         <v>66.501</v>
@@ -18923,7 +18933,7 @@
     </row>
     <row r="278">
       <c r="A278" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B278" s="2" t="n">
         <v>47.89</v>
@@ -18982,7 +18992,7 @@
     </row>
     <row r="279">
       <c r="A279" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B279" s="2" t="n">
         <v>38.231</v>
@@ -19041,7 +19051,7 @@
     </row>
     <row r="280">
       <c r="A280" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B280" s="2" t="n">
         <v>65.916</v>
@@ -19100,7 +19110,7 @@
     </row>
     <row r="281">
       <c r="A281" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B281" s="2" t="n">
         <v>60.358</v>
@@ -19159,7 +19169,7 @@
     </row>
     <row r="282">
       <c r="A282" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B282" s="2" t="n">
         <v>75.24</v>
@@ -19218,7 +19228,7 @@
     </row>
     <row r="283">
       <c r="A283" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B283" s="2" t="n">
         <v>62.321</v>
@@ -19277,7 +19287,7 @@
     </row>
     <row r="284">
       <c r="A284" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B284" s="2" t="n">
         <v>94.266</v>
@@ -19336,7 +19346,7 @@
     </row>
     <row r="285">
       <c r="A285" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B285" s="2" t="n">
         <v>60.362</v>
@@ -19395,7 +19405,7 @@
     </row>
     <row r="286">
       <c r="A286" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B286" s="2" t="n">
         <v>72.259</v>
@@ -19454,7 +19464,7 @@
     </row>
     <row r="287">
       <c r="A287" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B287" s="2" t="n">
         <v>98.75</v>
@@ -19513,7 +19523,7 @@
     </row>
     <row r="288">
       <c r="A288" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B288" s="2" t="n">
         <v>54.725</v>
@@ -19572,7 +19582,7 @@
     </row>
     <row r="289">
       <c r="A289" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B289" s="2" t="n">
         <v>70.776</v>
@@ -19631,7 +19641,7 @@
     </row>
     <row r="290">
       <c r="A290" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B290" s="2" t="n">
         <v>68.453</v>
@@ -19690,7 +19700,7 @@
     </row>
     <row r="291">
       <c r="A291" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B291" s="2" t="n">
         <v>53.693</v>
@@ -19749,7 +19759,7 @@
     </row>
     <row r="292">
       <c r="A292" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B292" s="2" t="n">
         <v>83.679</v>
@@ -19808,7 +19818,7 @@
     </row>
     <row r="293">
       <c r="A293" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B293" s="2" t="n">
         <v>47.896</v>
@@ -19867,7 +19877,7 @@
     </row>
     <row r="294">
       <c r="A294" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B294" s="2" t="n">
         <v>61.056</v>
@@ -19926,7 +19936,7 @@
     </row>
     <row r="295">
       <c r="A295" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B295" s="2" t="n">
         <v>70.446</v>
@@ -19985,7 +19995,7 @@
     </row>
     <row r="296">
       <c r="A296" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B296" s="2" t="n">
         <v>77.294</v>
@@ -20044,7 +20054,7 @@
     </row>
     <row r="297">
       <c r="A297" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B297" s="2" t="n">
         <v>76.133</v>
@@ -20103,7 +20113,7 @@
     </row>
     <row r="298">
       <c r="A298" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B298" s="2" t="n">
         <v>75.716</v>
@@ -20162,7 +20172,7 @@
     </row>
     <row r="299">
       <c r="A299" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B299" s="2" t="n">
         <v>92.13</v>
@@ -20221,7 +20231,7 @@
     </row>
     <row r="300">
       <c r="A300" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B300" s="2" t="n">
         <v>64.014</v>
@@ -20280,7 +20290,7 @@
     </row>
     <row r="301">
       <c r="A301" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B301" s="2" t="n">
         <v>45.697</v>
@@ -20339,7 +20349,7 @@
     </row>
     <row r="302">
       <c r="A302" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B302" s="2" t="n">
         <v>34.497</v>
@@ -20398,7 +20408,7 @@
     </row>
     <row r="303">
       <c r="A303" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B303" s="2" t="n">
         <v>61.145</v>
@@ -20457,7 +20467,7 @@
     </row>
     <row r="304">
       <c r="A304" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B304" s="2" t="n">
         <v>61.002</v>
@@ -20516,7 +20526,7 @@
     </row>
     <row r="305">
       <c r="A305" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B305" s="2" t="n">
         <v>64.585</v>
@@ -20575,7 +20585,7 @@
     </row>
     <row r="306">
       <c r="A306" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B306" s="2" t="n">
         <v>67.195</v>
@@ -20634,7 +20644,7 @@
     </row>
     <row r="307">
       <c r="A307" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B307" s="2" t="n">
         <v>77.349</v>
@@ -20693,7 +20703,7 @@
     </row>
     <row r="308">
       <c r="A308" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B308" s="2" t="n">
         <v>45.849</v>
@@ -20752,7 +20762,7 @@
     </row>
     <row r="309">
       <c r="A309" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B309" s="2" t="n">
         <v>42.208</v>
@@ -20811,7 +20821,7 @@
     </row>
     <row r="310">
       <c r="A310" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B310" s="2" t="n">
         <v>49.928</v>
@@ -20870,7 +20880,7 @@
     </row>
     <row r="311">
       <c r="A311" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B311" s="2" t="n">
         <v>53.104</v>
@@ -20929,7 +20939,7 @@
     </row>
     <row r="312">
       <c r="A312" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B312" s="2" t="n">
         <v>42.98</v>
@@ -20988,7 +20998,7 @@
     </row>
     <row r="313">
       <c r="A313" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B313" s="2" t="n">
         <v>57.54</v>
@@ -21047,7 +21057,7 @@
     </row>
     <row r="314">
       <c r="A314" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B314" s="2" t="n">
         <v>55.312</v>
@@ -21106,7 +21116,7 @@
     </row>
     <row r="315">
       <c r="A315" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B315" s="2" t="n">
         <v>46.279</v>
@@ -21165,7 +21175,7 @@
     </row>
     <row r="316">
       <c r="A316" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B316" s="2" t="n">
         <v>47.111</v>
@@ -21224,7 +21234,7 @@
     </row>
     <row r="317">
       <c r="A317" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B317" s="2" t="n">
         <v>70.968</v>
@@ -21283,7 +21293,7 @@
     </row>
     <row r="318">
       <c r="A318" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B318" s="2" t="n">
         <v>55.366</v>
@@ -21342,7 +21352,7 @@
     </row>
     <row r="319">
       <c r="A319" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B319" s="2" t="n">
         <v>52.582</v>
@@ -21401,7 +21411,7 @@
     </row>
     <row r="320">
       <c r="A320" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B320" s="2" t="n">
         <v>43.159</v>
@@ -21460,7 +21470,7 @@
     </row>
     <row r="321">
       <c r="A321" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B321" s="2" t="n">
         <v>53.071</v>
@@ -21519,7 +21529,7 @@
     </row>
     <row r="322">
       <c r="A322" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="B322" s="2" t="n">
         <v>57.323</v>
@@ -21578,7 +21588,7 @@
     </row>
     <row r="323">
       <c r="A323" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B323" s="2" t="n">
         <v>50.858</v>
@@ -21637,7 +21647,7 @@
     </row>
     <row r="324">
       <c r="A324" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="B324" s="2" t="n">
         <v>48.602</v>
@@ -21696,7 +21706,7 @@
     </row>
     <row r="325">
       <c r="A325" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B325" s="2" t="n">
         <v>43.908</v>
@@ -21755,7 +21765,7 @@
     </row>
     <row r="326">
       <c r="A326" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="B326" s="2" t="n">
         <v>40.647</v>
@@ -21814,7 +21824,7 @@
     </row>
     <row r="327">
       <c r="A327" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B327" s="2" t="n">
         <v>44.565</v>
@@ -21873,7 +21883,7 @@
     </row>
     <row r="328">
       <c r="A328" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="B328" s="2" t="n">
         <v>44.653</v>
@@ -21932,7 +21942,7 @@
     </row>
     <row r="329">
       <c r="A329" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B329" s="2" t="n">
         <v>44.731</v>
@@ -21991,7 +22001,7 @@
     </row>
     <row r="330">
       <c r="A330" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="B330" s="2" t="n">
         <v>50.135</v>
@@ -22050,7 +22060,7 @@
     </row>
     <row r="331">
       <c r="A331" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B331" s="2" t="n">
         <v>56.101</v>
@@ -22109,7 +22119,7 @@
     </row>
     <row r="332">
       <c r="A332" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="B332" s="2" t="n">
         <v>52.36</v>
@@ -22168,7 +22178,7 @@
     </row>
     <row r="333">
       <c r="A333" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="B333" s="2" t="n">
         <v>42.083</v>
@@ -22227,7 +22237,7 @@
     </row>
     <row r="334">
       <c r="A334" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="B334" s="2" t="n">
         <v>45.557</v>
@@ -22286,7 +22296,7 @@
     </row>
     <row r="335">
       <c r="A335" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="B335" s="2" t="n">
         <v>55.991</v>
@@ -22345,7 +22355,7 @@
     </row>
     <row r="336">
       <c r="A336" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="B336" s="2" t="n">
         <v>43.787</v>
@@ -22404,7 +22414,7 @@
     </row>
     <row r="337">
       <c r="A337" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="B337" s="2" t="n">
         <v>55.186</v>
@@ -22463,7 +22473,7 @@
     </row>
     <row r="338">
       <c r="A338" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="B338" s="2" t="n">
         <v>37.595</v>
@@ -22522,7 +22532,7 @@
     </row>
     <row r="339">
       <c r="A339" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="B339" s="2" t="n">
         <v>33.938</v>
@@ -22581,7 +22591,7 @@
     </row>
     <row r="340">
       <c r="A340" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="B340" s="2" t="n">
         <v>38.666</v>
@@ -22640,7 +22650,7 @@
     </row>
     <row r="341">
       <c r="A341" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="B341" s="2" t="n">
         <v>57.023</v>
@@ -22699,7 +22709,7 @@
     </row>
     <row r="342">
       <c r="A342" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="B342" s="2" t="n">
         <v>42.965</v>
@@ -22758,7 +22768,7 @@
     </row>
     <row r="343">
       <c r="A343" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="B343" s="2" t="n">
         <v>40.443</v>
@@ -22817,7 +22827,7 @@
     </row>
     <row r="344">
       <c r="A344" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="B344" s="2" t="n">
         <v>83.948</v>
@@ -22876,7 +22886,7 @@
     </row>
     <row r="345">
       <c r="A345" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="B345" s="2" t="n">
         <v>52.604</v>
@@ -22935,7 +22945,7 @@
     </row>
     <row r="346">
       <c r="A346" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="B346" s="2" t="n">
         <v>57.795</v>
@@ -22994,7 +23004,7 @@
     </row>
     <row r="347">
       <c r="A347" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="B347" s="2" t="n">
         <v>60.193</v>
@@ -23053,7 +23063,7 @@
     </row>
     <row r="348">
       <c r="A348" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="B348" s="2" t="n">
         <v>41.367</v>
@@ -23112,7 +23122,7 @@
     </row>
     <row r="349">
       <c r="A349" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="B349" s="2" t="n">
         <v>61.664</v>
@@ -23171,7 +23181,7 @@
     </row>
     <row r="350">
       <c r="A350" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="B350" s="2" t="n">
         <v>41.758</v>
@@ -23230,7 +23240,7 @@
     </row>
     <row r="351">
       <c r="A351" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="B351" s="2" t="n">
         <v>39.075</v>
@@ -23289,7 +23299,7 @@
     </row>
     <row r="352">
       <c r="A352" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B352" s="2" t="n">
         <v>31.27</v>
@@ -23348,7 +23358,7 @@
     </row>
     <row r="353">
       <c r="A353" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="B353" s="2" t="n">
         <v>3.19</v>
@@ -23407,7 +23417,7 @@
     </row>
     <row r="354">
       <c r="A354" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="B354" s="2" t="n">
         <v>29.012</v>
@@ -23466,7 +23476,7 @@
     </row>
     <row r="355">
       <c r="A355" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B355" s="2" t="n">
         <v>28.071</v>
@@ -23525,7 +23535,7 @@
     </row>
     <row r="356">
       <c r="A356" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="B356" s="2" t="n">
         <v>39.877</v>
@@ -23584,7 +23594,7 @@
     </row>
     <row r="357">
       <c r="A357" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B357" s="2" t="n">
         <v>34.678</v>
@@ -23643,7 +23653,7 @@
     </row>
     <row r="358">
       <c r="A358" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="B358" s="2" t="n">
         <v>32.426</v>
@@ -23702,7 +23712,7 @@
     </row>
     <row r="359">
       <c r="A359" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="B359" s="2" t="n">
         <v>50.689</v>
@@ -23761,7 +23771,7 @@
     </row>
     <row r="360">
       <c r="A360" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="B360" s="2" t="n">
         <v>51.334</v>
@@ -23820,7 +23830,7 @@
     </row>
     <row r="361">
       <c r="A361" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B361" s="2" t="n">
         <v>44.2</v>
@@ -23879,7 +23889,7 @@
     </row>
     <row r="362">
       <c r="A362" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="B362" s="2" t="n">
         <v>66.761</v>
@@ -23938,7 +23948,7 @@
     </row>
     <row r="363">
       <c r="A363" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B363" s="2" t="n">
         <v>35.433</v>
@@ -23997,7 +24007,7 @@
     </row>
     <row r="364">
       <c r="A364" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B364" s="2" t="n">
         <v>45.36</v>
@@ -24056,7 +24066,7 @@
     </row>
     <row r="365">
       <c r="A365" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="B365" s="2" t="n">
         <v>38.343</v>
@@ -24115,7 +24125,7 @@
     </row>
     <row r="366">
       <c r="A366" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="B366" s="2" t="n">
         <v>49.307</v>
@@ -24174,7 +24184,7 @@
     </row>
     <row r="367">
       <c r="A367" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="B367" s="2" t="n">
         <v>66.79</v>
@@ -24233,7 +24243,7 @@
     </row>
     <row r="368">
       <c r="A368" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="B368" s="2" t="n">
         <v>48.081</v>
@@ -24292,7 +24302,7 @@
     </row>
     <row r="369">
       <c r="A369" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="B369" s="2" t="n">
         <v>50.996</v>
@@ -24351,7 +24361,7 @@
     </row>
     <row r="370">
       <c r="A370" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="B370" s="2" t="n">
         <v>38.723</v>
@@ -24410,7 +24420,7 @@
     </row>
     <row r="371">
       <c r="A371" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="B371" s="2" t="n">
         <v>36.33</v>
@@ -24469,7 +24479,7 @@
     </row>
     <row r="372">
       <c r="A372" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="B372" s="2" t="n">
         <v>32.382</v>
@@ -24528,7 +24538,7 @@
     </row>
     <row r="373">
       <c r="A373" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B373" s="2" t="n">
         <v>55.558</v>
@@ -24587,7 +24597,7 @@
     </row>
     <row r="374">
       <c r="A374" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="B374" s="2" t="n">
         <v>32.868</v>
@@ -24646,7 +24656,7 @@
     </row>
     <row r="375">
       <c r="A375" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="B375" s="2" t="n">
         <v>50.915</v>
@@ -24705,7 +24715,7 @@
     </row>
     <row r="376">
       <c r="A376" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="B376" s="2" t="n">
         <v>37.357</v>
@@ -24764,7 +24774,7 @@
     </row>
     <row r="377">
       <c r="A377" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="B377" s="2" t="n">
         <v>55.236</v>
@@ -24823,7 +24833,7 @@
     </row>
     <row r="378">
       <c r="A378" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="B378" s="2" t="n">
         <v>67.728</v>
@@ -24882,7 +24892,7 @@
     </row>
     <row r="379">
       <c r="A379" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="B379" s="2" t="n">
         <v>47.705</v>
@@ -24941,7 +24951,7 @@
     </row>
     <row r="380">
       <c r="A380" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="B380" s="2" t="n">
         <v>41.112</v>
@@ -25000,7 +25010,7 @@
     </row>
     <row r="381">
       <c r="A381" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="B381" s="2" t="n">
         <v>43.674</v>
@@ -25059,7 +25069,7 @@
     </row>
     <row r="382">
       <c r="A382" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="B382" s="2" t="n">
         <v>60.069</v>
@@ -25118,7 +25128,7 @@
     </row>
     <row r="383">
       <c r="A383" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="B383" s="2" t="n">
         <v>43.887</v>
@@ -25177,7 +25187,7 @@
     </row>
     <row r="384">
       <c r="A384" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="B384" s="2" t="n">
         <v>70.605</v>
@@ -25236,7 +25246,7 @@
     </row>
     <row r="385">
       <c r="A385" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="B385" s="2" t="n">
         <v>41.307</v>
@@ -25295,7 +25305,7 @@
     </row>
     <row r="386">
       <c r="A386" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="B386" s="2" t="n">
         <v>51.802</v>
@@ -25354,7 +25364,7 @@
     </row>
     <row r="387">
       <c r="A387" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="B387" s="2" t="n">
         <v>53.241</v>
@@ -25413,7 +25423,7 @@
     </row>
     <row r="388">
       <c r="A388" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="B388" s="2" t="n">
         <v>63.902</v>
@@ -25472,7 +25482,7 @@
     </row>
     <row r="389">
       <c r="A389" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B389" s="2" t="n">
         <v>33.032</v>
@@ -25531,7 +25541,7 @@
     </row>
     <row r="390">
       <c r="A390" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="B390" s="2" t="n">
         <v>37.262</v>
@@ -25590,7 +25600,7 @@
     </row>
     <row r="391">
       <c r="A391" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="B391" s="2" t="n">
         <v>51.347</v>
@@ -25649,7 +25659,7 @@
     </row>
     <row r="392">
       <c r="A392" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="B392" s="2" t="n">
         <v>54.374</v>
@@ -25708,7 +25718,7 @@
     </row>
     <row r="393">
       <c r="A393" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="B393" s="2" t="n">
         <v>66.663</v>
@@ -25767,7 +25777,7 @@
     </row>
     <row r="394">
       <c r="A394" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="B394" s="2" t="n">
         <v>58.488</v>
@@ -25826,7 +25836,7 @@
     </row>
     <row r="395">
       <c r="A395" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B395" s="2" t="n">
         <v>29.971</v>
@@ -25885,7 +25895,7 @@
     </row>
     <row r="396">
       <c r="A396" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="B396" s="2" t="n">
         <v>35.244</v>
@@ -25944,7 +25954,7 @@
     </row>
     <row r="397">
       <c r="A397" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="B397" s="2" t="n">
         <v>56.269</v>
@@ -26003,7 +26013,7 @@
     </row>
     <row r="398">
       <c r="A398" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="B398" s="2" t="n">
         <v>24.795</v>
@@ -26062,7 +26072,7 @@
     </row>
     <row r="399">
       <c r="A399" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="B399" s="2" t="n">
         <v>21.802</v>
@@ -26121,7 +26131,7 @@
     </row>
     <row r="400">
       <c r="A400" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="B400" s="2" t="n">
         <v>32.552</v>
@@ -26180,7 +26190,7 @@
     </row>
     <row r="401">
       <c r="A401" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="B401" s="2" t="n">
         <v>38.154</v>
@@ -26239,7 +26249,7 @@
     </row>
     <row r="402">
       <c r="A402" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="B402" s="2" t="n">
         <v>26.071</v>
@@ -26298,7 +26308,7 @@
     </row>
     <row r="403">
       <c r="A403" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="B403" s="2" t="n">
         <v>26.604</v>
@@ -26357,7 +26367,7 @@
     </row>
     <row r="404">
       <c r="A404" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="B404" s="2" t="n">
         <v>32.745</v>
@@ -26416,7 +26426,7 @@
     </row>
     <row r="405">
       <c r="A405" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="B405" s="2" t="n">
         <v>40.745</v>
@@ -26475,7 +26485,7 @@
     </row>
     <row r="406">
       <c r="A406" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="B406" s="2" t="n">
         <v>51.901</v>
@@ -26534,7 +26544,7 @@
     </row>
     <row r="407">
       <c r="A407" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="B407" s="2" t="n">
         <v>70.643</v>
@@ -26593,7 +26603,7 @@
     </row>
     <row r="408">
       <c r="A408" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="B408" s="2" t="n">
         <v>32.522</v>
@@ -26652,7 +26662,7 @@
     </row>
     <row r="409">
       <c r="A409" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="B409" s="2" t="n">
         <v>66.591</v>
@@ -26711,7 +26721,7 @@
     </row>
     <row r="410">
       <c r="A410" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B410" s="2" t="n">
         <v>30.425</v>
@@ -26770,7 +26780,7 @@
     </row>
     <row r="411">
       <c r="A411" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="B411" s="2" t="n">
         <v>34.472</v>
@@ -26829,7 +26839,7 @@
     </row>
     <row r="412">
       <c r="A412" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="B412" s="2" t="n">
         <v>36.967</v>
@@ -26888,7 +26898,7 @@
     </row>
     <row r="413">
       <c r="A413" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="B413" s="2" t="n">
         <v>29.735</v>
@@ -26947,7 +26957,7 @@
     </row>
     <row r="414">
       <c r="A414" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="B414" s="2" t="n">
         <v>42.018</v>
@@ -27006,7 +27016,7 @@
     </row>
     <row r="415">
       <c r="A415" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="B415" s="2" t="n">
         <v>39.332</v>
@@ -27065,7 +27075,7 @@
     </row>
     <row r="416">
       <c r="A416" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="B416" s="2" t="n">
         <v>43.288</v>
@@ -27124,7 +27134,7 @@
     </row>
     <row r="417">
       <c r="A417" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="B417" s="2" t="n">
         <v>41.319</v>
@@ -27183,7 +27193,7 @@
     </row>
     <row r="418">
       <c r="A418" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="B418" s="2" t="n">
         <v>38.487</v>
@@ -27242,7 +27252,7 @@
     </row>
     <row r="419">
       <c r="A419" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="B419" s="2" t="n">
         <v>70.544</v>
@@ -27301,7 +27311,7 @@
     </row>
     <row r="420">
       <c r="A420" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="B420" s="2" t="n">
         <v>41.589</v>
@@ -27360,7 +27370,7 @@
     </row>
     <row r="421">
       <c r="A421" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="B421" s="2" t="n">
         <v>45.879</v>
@@ -27419,7 +27429,7 @@
     </row>
     <row r="422">
       <c r="A422" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="B422" s="2" t="n">
         <v>37.859</v>
@@ -27478,7 +27488,7 @@
     </row>
     <row r="423">
       <c r="A423" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="B423" s="2" t="n">
         <v>38.555</v>
@@ -27537,7 +27547,7 @@
     </row>
     <row r="424">
       <c r="A424" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="B424" s="2" t="n">
         <v>43.01</v>
@@ -27596,7 +27606,7 @@
     </row>
     <row r="425">
       <c r="A425" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B425" s="2" t="n">
         <v>37.776</v>
@@ -27655,7 +27665,7 @@
     </row>
     <row r="426">
       <c r="A426" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="B426" s="2"/>
       <c r="C426" s="3" t="n">
@@ -27688,7 +27698,7 @@
     </row>
     <row r="427">
       <c r="A427" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="B427" s="2"/>
       <c r="C427" s="3" t="n">
@@ -27721,7 +27731,7 @@
     </row>
     <row r="428">
       <c r="A428" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="B428" s="2"/>
       <c r="C428" s="3" t="n">
@@ -27754,7 +27764,7 @@
     </row>
     <row r="429">
       <c r="A429" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="B429" s="2"/>
       <c r="C429" s="3" t="n">
@@ -27787,7 +27797,7 @@
     </row>
     <row r="430">
       <c r="A430" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="B430" s="2"/>
       <c r="C430" s="3" t="n">
@@ -27820,7 +27830,7 @@
     </row>
     <row r="431">
       <c r="A431" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="B431" s="2"/>
       <c r="C431" s="3" t="n">
@@ -27853,7 +27863,7 @@
     </row>
     <row r="432">
       <c r="A432" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="B432" s="2"/>
       <c r="C432" s="3" t="n">
@@ -27886,7 +27896,7 @@
     </row>
     <row r="433">
       <c r="A433" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="B433" s="2"/>
       <c r="C433" s="3" t="n">
@@ -27919,7 +27929,7 @@
     </row>
     <row r="434">
       <c r="A434" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="B434" s="2"/>
       <c r="C434" s="3" t="n">
@@ -27952,7 +27962,7 @@
     </row>
     <row r="435">
       <c r="A435" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="B435" s="2"/>
       <c r="C435" s="3" t="n">
@@ -27985,7 +27995,7 @@
     </row>
     <row r="436">
       <c r="A436" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="B436" s="2"/>
       <c r="C436" s="3" t="n">
@@ -28018,7 +28028,7 @@
     </row>
     <row r="437">
       <c r="A437" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="B437" s="2"/>
       <c r="C437" s="3" t="n">
@@ -28051,7 +28061,7 @@
     </row>
     <row r="438">
       <c r="A438" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="B438" s="2"/>
       <c r="C438" s="3"/>
@@ -28074,7 +28084,7 @@
     </row>
     <row r="439">
       <c r="A439" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="B439" s="2"/>
       <c r="C439" s="3"/>
@@ -28097,7 +28107,7 @@
     </row>
     <row r="440">
       <c r="A440" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="B440" s="2"/>
       <c r="C440" s="3"/>
@@ -28120,7 +28130,7 @@
     </row>
     <row r="441">
       <c r="A441" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="B441" s="2"/>
       <c r="C441" s="3"/>
@@ -28143,7 +28153,7 @@
     </row>
     <row r="442">
       <c r="A442" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="B442" s="2"/>
       <c r="C442" s="3"/>
@@ -28166,7 +28176,7 @@
     </row>
     <row r="443">
       <c r="A443" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="B443" s="2"/>
       <c r="C443" s="3"/>
@@ -28189,7 +28199,7 @@
     </row>
     <row r="444">
       <c r="A444" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="B444" s="2"/>
       <c r="C444" s="3"/>
@@ -28212,7 +28222,7 @@
     </row>
     <row r="445">
       <c r="A445" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="B445" s="2"/>
       <c r="C445" s="3"/>
@@ -28235,7 +28245,7 @@
     </row>
     <row r="446">
       <c r="A446" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="B446" s="2"/>
       <c r="C446" s="3"/>
@@ -28258,7 +28268,7 @@
     </row>
     <row r="447">
       <c r="A447" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="B447" s="2"/>
       <c r="C447" s="3"/>
@@ -28281,7 +28291,7 @@
     </row>
     <row r="448">
       <c r="A448" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="B448" s="2"/>
       <c r="C448" s="3"/>
@@ -28304,7 +28314,7 @@
     </row>
     <row r="449">
       <c r="A449" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="B449" s="2"/>
       <c r="C449" s="3"/>
@@ -28327,7 +28337,7 @@
     </row>
     <row r="450">
       <c r="A450" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="B450" s="2"/>
       <c r="C450" s="3"/>
@@ -28350,7 +28360,7 @@
     </row>
     <row r="451">
       <c r="A451" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="B451" s="2"/>
       <c r="C451" s="3"/>
@@ -28373,7 +28383,7 @@
     </row>
     <row r="452">
       <c r="A452" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="B452" s="2"/>
       <c r="C452" s="3"/>
@@ -28396,7 +28406,7 @@
     </row>
     <row r="453">
       <c r="A453" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="B453" s="2"/>
       <c r="C453" s="3"/>
@@ -28419,7 +28429,7 @@
     </row>
     <row r="454">
       <c r="A454" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="B454" s="2"/>
       <c r="C454" s="3"/>
@@ -28442,7 +28452,7 @@
     </row>
     <row r="455">
       <c r="A455" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="B455" s="2"/>
       <c r="C455" s="3"/>
@@ -28465,7 +28475,7 @@
     </row>
     <row r="456">
       <c r="A456" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="B456" s="2"/>
       <c r="C456" s="3"/>
@@ -28488,7 +28498,7 @@
     </row>
     <row r="457">
       <c r="A457" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="B457" s="2"/>
       <c r="C457" s="3"/>
@@ -28511,7 +28521,7 @@
     </row>
     <row r="458">
       <c r="A458" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="B458" s="2"/>
       <c r="C458" s="3"/>
@@ -28534,7 +28544,7 @@
     </row>
     <row r="459">
       <c r="A459" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="B459" s="2"/>
       <c r="C459" s="3"/>
@@ -28557,7 +28567,7 @@
     </row>
     <row r="460">
       <c r="A460" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="B460" s="2"/>
       <c r="C460" s="3"/>
@@ -28580,7 +28590,7 @@
     </row>
     <row r="461">
       <c r="A461" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="B461" s="2"/>
       <c r="C461" s="3"/>
@@ -28603,7 +28613,7 @@
     </row>
     <row r="462">
       <c r="A462" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="B462" s="2"/>
       <c r="C462" s="3"/>
@@ -28626,7 +28636,7 @@
     </row>
     <row r="463">
       <c r="A463" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="B463" s="2"/>
       <c r="C463" s="3"/>
@@ -28649,7 +28659,7 @@
     </row>
     <row r="464">
       <c r="A464" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="B464" s="2"/>
       <c r="C464" s="3"/>
@@ -28672,7 +28682,7 @@
     </row>
     <row r="465">
       <c r="A465" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="B465" s="2"/>
       <c r="C465" s="3"/>
@@ -28695,7 +28705,7 @@
     </row>
     <row r="466">
       <c r="A466" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="B466" s="2"/>
       <c r="C466" s="3"/>
@@ -28718,7 +28728,7 @@
     </row>
     <row r="467">
       <c r="A467" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="B467" s="2"/>
       <c r="C467" s="3"/>
@@ -28741,7 +28751,7 @@
     </row>
     <row r="468">
       <c r="A468" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="B468" s="2"/>
       <c r="C468" s="3"/>
@@ -28764,7 +28774,7 @@
     </row>
     <row r="469">
       <c r="A469" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="B469" s="2"/>
       <c r="C469" s="3"/>
@@ -28787,7 +28797,7 @@
     </row>
     <row r="470">
       <c r="A470" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="B470" s="2"/>
       <c r="C470" s="3"/>
@@ -28810,7 +28820,7 @@
     </row>
     <row r="471">
       <c r="A471" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="B471" s="2"/>
       <c r="C471" s="3"/>
@@ -28833,7 +28843,7 @@
     </row>
     <row r="472">
       <c r="A472" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B472" s="2"/>
       <c r="C472" s="3"/>
@@ -28856,7 +28866,7 @@
     </row>
     <row r="473">
       <c r="A473" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="B473" s="2"/>
       <c r="C473" s="3"/>
@@ -28879,7 +28889,7 @@
     </row>
     <row r="474">
       <c r="A474" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="B474" s="2"/>
       <c r="C474" s="3"/>
@@ -28902,7 +28912,7 @@
     </row>
     <row r="475">
       <c r="A475" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="B475" s="2"/>
       <c r="C475" s="3"/>
@@ -28925,7 +28935,7 @@
     </row>
     <row r="476">
       <c r="A476" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="B476" s="2"/>
       <c r="C476" s="3"/>
@@ -28948,7 +28958,7 @@
     </row>
     <row r="477">
       <c r="A477" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="B477" s="2"/>
       <c r="C477" s="3"/>
@@ -28971,7 +28981,7 @@
     </row>
     <row r="478">
       <c r="A478" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="B478" s="2"/>
       <c r="C478" s="3"/>
@@ -28994,7 +29004,7 @@
     </row>
     <row r="479">
       <c r="A479" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="B479" s="2"/>
       <c r="C479" s="3"/>
@@ -29017,7 +29027,7 @@
     </row>
     <row r="480">
       <c r="A480" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="B480" s="2"/>
       <c r="C480" s="3"/>
@@ -29040,7 +29050,7 @@
     </row>
     <row r="481">
       <c r="A481" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="B481" s="2"/>
       <c r="C481" s="3"/>
@@ -29074,97 +29084,97 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
   </sheetData>
@@ -29188,7 +29198,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -29198,13 +29208,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>0.016900786588572</v>
@@ -29212,7 +29222,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>0.0403835832167981</v>
@@ -29220,7 +29230,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>0.0768620630025475</v>
@@ -29228,7 +29238,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>0.0423821746392974</v>
@@ -29236,7 +29246,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>0.0350152737397484</v>
@@ -29244,7 +29254,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>0.0630012892807105</v>
@@ -29252,7 +29262,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>0.0546992032877723</v>
@@ -29260,7 +29270,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>0.0997390840810099</v>
@@ -29268,7 +29278,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>0.184461577556816</v>
@@ -29276,7 +29286,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>0.175095464493619</v>
@@ -29284,7 +29294,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>0.172769601053398</v>
@@ -29292,7 +29302,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>0.193003713127476</v>
@@ -29300,7 +29310,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>0.156008166580868</v>
@@ -29308,7 +29318,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>0.131443726233381</v>
@@ -29316,7 +29326,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>0.0871568625751816</v>
@@ -29324,7 +29334,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>-0.0333589953155873</v>
@@ -29332,7 +29342,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>-0.062805613681069</v>
@@ -29340,7 +29350,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>0.0113127342385974</v>
@@ -29348,7 +29358,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>-0.000335810186478149</v>

</xml_diff>